<commit_message>
Updated .xlsx file for testing this project
</commit_message>
<xml_diff>
--- a/example.xlsx
+++ b/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PYTHON_PROJECTS\Tender_Parcing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C594E0D-82A8-4158-B659-74604417B7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{788BE42A-02C1-4CE0-85D8-6C1E2DF94DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Name</t>
   </si>
@@ -37,6 +37,18 @@
   </si>
   <si>
     <t>Availability</t>
+  </si>
+  <si>
+    <t>MSI 27</t>
+  </si>
+  <si>
+    <t>MSI laptop 24</t>
+  </si>
+  <si>
+    <t>Huawei MatePad</t>
+  </si>
+  <si>
+    <t>Apple Ipad</t>
   </si>
 </sst>
 </file>
@@ -373,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -394,6 +406,26 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>